<commit_message>
Jar prompts: 20 more shapes (28 total)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/jar-prompts.xlsx
+++ b/docs/jar-prompts.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -652,6 +652,446 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>jar-milkcarton.png</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>กล่องนมใส</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass milk carton with a pink strawberry label shape outline and a folded pink top, empty inside</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass milk carton with a pink strawberry label shape outline and a folded pink top, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>jar-lantern.png</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>โคมไฟจีนใส</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass Chinese lantern with red-gold top and bottom caps and a tassel, empty glowing inside</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass Chinese lantern with red-gold top and bottom caps and a tassel, empty glowing inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>jar-perfume.png</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>ขวดน้ำหอม</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>a big heart-cut crystal perfume bottle with a pink bow and a gold atomizer pump, empty inside</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a big heart-cut crystal perfume bottle with a pink bow and a gold atomizer pump, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>jar-teapot.png</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>กาน้ำชาแก้ว</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>a round clear glass teapot with a pastel pink lid and spout, little flowers painted on the handle, empty inside</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a round clear glass teapot with a pastel pink lid and spout, little flowers painted on the handle, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>jar-hourglass.png</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>นาฬิกาทราย</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>a tall pastel hourglass with gold frame and two clear glass bulbs, empty inside</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a tall pastel hourglass with gold frame and two clear glass bulbs, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>jar-crown.png</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>มงกุฎแก้ว</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>a big clear glass crown-shaped jar with pink jewels on the tips and a gold base, empty inside</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a big clear glass crown-shaped jar with pink jewels on the tips and a gold base, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>jar-cupcake.png</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>คัพเค้กใส</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>a giant cupcake-shaped clear jar, pink wrapper base with ruffles, clear glass top shaped like swirled frosting, empty inside</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a giant cupcake-shaped clear jar, pink wrapper base with ruffles, clear glass top shaped like swirled frosting, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>jar-strawberry.png</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>ขวดสตรอว์เบอร์รี่</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass jar shaped like a strawberry with a green leafy lid, tiny seed dots on the glass, empty inside</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass jar shaped like a strawberry with a green leafy lid, tiny seed dots on the glass, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>jar-diamond.png</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>เพชรยักษ์</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>a giant faceted diamond-shaped clear glass container standing on a pink velvet cushion, opening at the top, empty inside</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a giant faceted diamond-shaped clear glass container standing on a pink velvet cushion, opening at the top, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>jar-piggybank.png</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>กระปุกหมูแก้ว</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass piggy bank with a pink snout, ears and feet, a coin slot on top, empty inside</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass piggy bank with a pink snout, ears and feet, a coin slot on top, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>jar-microphone.png</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>ไมค์ยักษ์</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>a giant karaoke microphone with a clear glass mesh head (hollow), pink and gold handle, empty inside the head</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a giant karaoke microphone with a clear glass mesh head (hollow), pink and gold handle, empty inside the head.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>jar-gamecontroller.png</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>จอยเกมใส</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>a big clear game console controller shaped container with pastel buttons, cyber neon pink-cyan edges, empty inside</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a big clear game console controller shaped container with pastel buttons, cyber neon pink-cyan edges, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>jar-robotcapsule.png</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>แคปซูลหุ่นยนต์</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>a futuristic cyber capsule pod with a clear glass window, black frame with neon cyan and pink lights, empty inside</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a futuristic cyber capsule pod with a clear glass window, black frame with neon cyan and pink lights, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>jar-treasure.png</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>หีบสมบัติแก้ว</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>an open treasure chest made of clear glass with gold trim and pink gems, lid open at the back, empty inside</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: an open treasure chest made of clear glass with gold trim and pink gems, lid open at the back, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>jar-snowman.png</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>มนุษย์หิมะแก้ว</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass snowman made of two stacked glass spheres, knitted pink hat and scarf, empty inside</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass snowman made of two stacked glass spheres, knitted pink hat and scarf, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>jar-pumpkin.png</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>ฟักทองแก้ว</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass pumpkin jar with a pastel orange stem lid and tiny bat stickers, empty inside</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass pumpkin jar with a pastel orange stem lid and tiny bat stickers, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>jar-sakura.png</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>ขวดซากุระ</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>a tall clear glass bottle with sakura branch painted around it, pink cork with a flower, empty inside</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a tall clear glass bottle with sakura branch painted around it, pink cork with a flower, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>jar-cloud.png</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ก้อนเมฆใส</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>a fluffy cloud-shaped clear glass container with a rainbow handle on top, tiny raindrop charms, empty inside</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a fluffy cloud-shaped clear glass container with a rainbow handle on top, tiny raindrop charms, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>jar-thaibowl.png</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>ขันน้ำไทย</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>a clear glass Thai silver-style water bowl (khan) with ornate gold Thai pattern rim, on a small pedestal, empty inside</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a clear glass Thai silver-style water bowl (khan) with ornate gold Thai pattern rim, on a small pedestal, empty inside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>jar-tuktuk.png</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>ตุ๊กตุ๊กใส</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>a cute Thai tuk-tuk with a clear glass passenger cabin, pink and gold body, empty inside the cabin</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Cute 3D pastel container for a TikTok LIVE gift overlay, soft glossy vinyl-toy style, smooth shading, clean outline, pink-lavender-mint palette, kawaii. Front view, centered, single object only. EMPTY inside — nothing inside, the inner space is clearly see-through clear glass/plastic so gifts can be added later. The glass must be very clear and colorless (no frosted or milky tint), with only a few thin highlight streaks on the edges. Transparent background, no shadow on ground, no text, 1024x1024. Object: a cute Thai tuk-tuk with a clear glass passenger cabin, pink and gold body, empty inside the cabin.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>

</xml_diff>